<commit_message>
update visualization and mapping code
</commit_message>
<xml_diff>
--- a/output/CS_SFIAFormat/sfiaformat_mapping_cosine_SkillNER QE_CS.xlsx
+++ b/output/CS_SFIAFormat/sfiaformat_mapping_cosine_SkillNER QE_CS.xlsx
@@ -480,16 +480,16 @@
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="n">
-        <v>0.2192</v>
+        <v>0.2643</v>
       </c>
       <c r="F2" t="n">
-        <v>0.3056</v>
+        <v>0.3706</v>
       </c>
       <c r="G2" t="n">
-        <v>0.2264</v>
+        <v>0.6477000000000001</v>
       </c>
       <c r="H2" t="n">
-        <v>0.2218</v>
+        <v>0.3553</v>
       </c>
     </row>
     <row r="3">
@@ -504,10 +504,10 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
-        <v>0.2603</v>
+        <v>0.3574</v>
       </c>
       <c r="H3" t="n">
-        <v>0.2426</v>
+        <v>0.368</v>
       </c>
     </row>
     <row r="4">
@@ -522,16 +522,16 @@
         <v>0.5901</v>
       </c>
       <c r="E4" t="n">
-        <v>0.3821</v>
+        <v>0.5903</v>
       </c>
       <c r="F4" t="n">
-        <v>0.2149</v>
+        <v>0.5212</v>
       </c>
       <c r="G4" t="n">
-        <v>0.2049</v>
+        <v>0.3343</v>
       </c>
       <c r="H4" t="n">
-        <v>0.2871</v>
+        <v>0.7175</v>
       </c>
     </row>
     <row r="5">
@@ -545,13 +545,13 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
-        <v>0.2836</v>
+        <v>0.5051</v>
       </c>
       <c r="G5" t="n">
-        <v>0.2155</v>
+        <v>0.2863</v>
       </c>
       <c r="H5" t="n">
-        <v>0.2022</v>
+        <v>0.2331</v>
       </c>
     </row>
     <row r="6">
@@ -564,13 +564,13 @@
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="n">
-        <v>0.2037</v>
+        <v>0.3627</v>
       </c>
       <c r="F6" t="n">
-        <v>0.212</v>
+        <v>0.4276</v>
       </c>
       <c r="G6" t="n">
-        <v>0.3092</v>
+        <v>0.4796</v>
       </c>
       <c r="H6" t="inlineStr"/>
     </row>
@@ -585,13 +585,13 @@
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
-        <v>0.2359</v>
+        <v>0.3263</v>
       </c>
       <c r="G7" t="n">
         <v>0.3162</v>
       </c>
       <c r="H7" t="n">
-        <v>0.2123</v>
+        <v>0.3482</v>
       </c>
     </row>
     <row r="8">
@@ -610,7 +610,7 @@
         <v>0.3074</v>
       </c>
       <c r="G8" t="n">
-        <v>0.2507</v>
+        <v>0.2922</v>
       </c>
       <c r="H8" t="inlineStr"/>
     </row>
@@ -623,16 +623,16 @@
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="n">
-        <v>0.2011</v>
+        <v>0.2947</v>
       </c>
       <c r="E9" t="n">
-        <v>0.2027</v>
+        <v>0.3239</v>
       </c>
       <c r="F9" t="n">
-        <v>0.2068</v>
+        <v>0.3477</v>
       </c>
       <c r="G9" t="n">
-        <v>0.2245</v>
+        <v>0.3662</v>
       </c>
       <c r="H9" t="inlineStr"/>
     </row>
@@ -664,13 +664,13 @@
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="n">
-        <v>0.259</v>
+        <v>0.5268</v>
       </c>
       <c r="F11" t="n">
-        <v>0.2054</v>
+        <v>0.4966</v>
       </c>
       <c r="G11" t="n">
-        <v>0.2144</v>
+        <v>0.4804</v>
       </c>
       <c r="H11" t="inlineStr"/>
     </row>
@@ -684,7 +684,7 @@
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="n">
-        <v>0.2173</v>
+        <v>0.3903</v>
       </c>
       <c r="F12" t="n">
         <v>0.221</v>
@@ -703,16 +703,16 @@
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="n">
-        <v>0.39</v>
+        <v>0.5294</v>
       </c>
       <c r="E13" t="n">
-        <v>0.2934</v>
+        <v>0.4035</v>
       </c>
       <c r="F13" t="n">
-        <v>0.2524</v>
+        <v>0.2783</v>
       </c>
       <c r="G13" t="n">
-        <v>0.2334</v>
+        <v>0.6143</v>
       </c>
       <c r="H13" t="inlineStr"/>
     </row>
@@ -727,13 +727,13 @@
         <v>0.3271</v>
       </c>
       <c r="D14" t="n">
-        <v>0.2551</v>
+        <v>0.3423</v>
       </c>
       <c r="E14" t="n">
         <v>0.3259</v>
       </c>
       <c r="F14" t="n">
-        <v>0.3533</v>
+        <v>0.3781</v>
       </c>
       <c r="G14" t="n">
         <v>0.3099</v>
@@ -748,16 +748,16 @@
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="n">
-        <v>0.2449</v>
+        <v>0.4664</v>
       </c>
       <c r="D15" t="n">
-        <v>0.2074</v>
+        <v>0.2968</v>
       </c>
       <c r="E15" t="n">
         <v>0.3336</v>
       </c>
       <c r="F15" t="n">
-        <v>0.2773</v>
+        <v>0.4193</v>
       </c>
       <c r="G15" t="n">
         <v>0.3556</v>
@@ -781,7 +781,7 @@
         <v>0.2985</v>
       </c>
       <c r="F16" t="n">
-        <v>0.2315</v>
+        <v>0.5441</v>
       </c>
       <c r="G16" t="n">
         <v>0.2003</v>
@@ -798,13 +798,13 @@
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="n">
-        <v>0.2829</v>
+        <v>0.4057</v>
       </c>
       <c r="F17" t="n">
-        <v>0.2454</v>
+        <v>0.4289</v>
       </c>
       <c r="G17" t="n">
-        <v>0.2037</v>
+        <v>0.4978</v>
       </c>
       <c r="H17" t="inlineStr"/>
     </row>
@@ -819,16 +819,16 @@
         <v>0.3565</v>
       </c>
       <c r="D18" t="n">
-        <v>0.274</v>
+        <v>0.3796</v>
       </c>
       <c r="E18" t="n">
-        <v>0.2259</v>
+        <v>0.4307</v>
       </c>
       <c r="F18" t="n">
-        <v>0.2878</v>
+        <v>0.5163</v>
       </c>
       <c r="G18" t="n">
-        <v>0.2215</v>
+        <v>0.4422</v>
       </c>
       <c r="H18" t="inlineStr"/>
     </row>
@@ -840,22 +840,22 @@
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="n">
-        <v>0.3215</v>
+        <v>0.391</v>
       </c>
       <c r="D19" t="n">
-        <v>0.2232</v>
+        <v>0.3241</v>
       </c>
       <c r="E19" t="n">
-        <v>0.2808</v>
+        <v>0.5296999999999999</v>
       </c>
       <c r="F19" t="n">
-        <v>0.3091</v>
+        <v>0.4879</v>
       </c>
       <c r="G19" t="n">
-        <v>0.2401</v>
+        <v>0.3141</v>
       </c>
       <c r="H19" t="n">
-        <v>0.2807</v>
+        <v>0.4064</v>
       </c>
     </row>
     <row r="20">
@@ -866,22 +866,22 @@
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="n">
-        <v>0.2658</v>
+        <v>0.5367</v>
       </c>
       <c r="D20" t="n">
-        <v>0.2104</v>
+        <v>0.5286999999999999</v>
       </c>
       <c r="E20" t="n">
-        <v>0.2788</v>
+        <v>0.4014</v>
       </c>
       <c r="F20" t="n">
-        <v>0.2819</v>
+        <v>0.4708</v>
       </c>
       <c r="G20" t="n">
-        <v>0.2508</v>
+        <v>0.4607</v>
       </c>
       <c r="H20" t="n">
-        <v>0.2847</v>
+        <v>0.523</v>
       </c>
     </row>
     <row r="21">
@@ -894,13 +894,13 @@
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="n">
-        <v>0.361</v>
+        <v>0.5561</v>
       </c>
       <c r="F21" t="n">
-        <v>0.238</v>
+        <v>0.6242</v>
       </c>
       <c r="G21" t="n">
-        <v>0.2441</v>
+        <v>0.4049</v>
       </c>
       <c r="H21" t="inlineStr"/>
     </row>
@@ -912,19 +912,19 @@
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="n">
-        <v>0.2138</v>
+        <v>0.2889</v>
       </c>
       <c r="D22" t="n">
-        <v>0.2221</v>
+        <v>0.3354</v>
       </c>
       <c r="E22" t="n">
-        <v>0.2478</v>
+        <v>0.4258</v>
       </c>
       <c r="F22" t="n">
-        <v>0.3092</v>
+        <v>0.351</v>
       </c>
       <c r="G22" t="n">
-        <v>0.2349</v>
+        <v>0.3831</v>
       </c>
       <c r="H22" t="inlineStr"/>
     </row>
@@ -937,16 +937,16 @@
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="n">
-        <v>0.2011</v>
+        <v>0.6579</v>
       </c>
       <c r="E23" t="n">
-        <v>0.2111</v>
+        <v>0.2636</v>
       </c>
       <c r="F23" t="n">
-        <v>0.2079</v>
+        <v>0.258</v>
       </c>
       <c r="G23" t="n">
-        <v>0.2517</v>
+        <v>0.2944</v>
       </c>
       <c r="H23" t="inlineStr"/>
     </row>
@@ -962,10 +962,10 @@
       <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="n">
-        <v>0.2614</v>
+        <v>0.326</v>
       </c>
       <c r="H24" t="n">
-        <v>0.2673</v>
+        <v>0.4164</v>
       </c>
     </row>
     <row r="25">
@@ -976,22 +976,22 @@
       </c>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="n">
-        <v>0.3109</v>
+        <v>0.4461</v>
       </c>
       <c r="D25" t="n">
-        <v>0.2612</v>
+        <v>0.468</v>
       </c>
       <c r="E25" t="n">
-        <v>0.3775</v>
+        <v>0.4512</v>
       </c>
       <c r="F25" t="n">
-        <v>0.2243</v>
+        <v>0.4194</v>
       </c>
       <c r="G25" t="n">
-        <v>0.2641</v>
+        <v>0.4343</v>
       </c>
       <c r="H25" t="n">
-        <v>0.2234</v>
+        <v>0.4651</v>
       </c>
     </row>
     <row r="26">
@@ -1003,16 +1003,16 @@
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="n">
-        <v>0.2419</v>
+        <v>0.2557</v>
       </c>
       <c r="E26" t="n">
-        <v>0.2003</v>
+        <v>0.4039</v>
       </c>
       <c r="F26" t="n">
-        <v>0.3145</v>
+        <v>0.4537</v>
       </c>
       <c r="G26" t="n">
-        <v>0.4031</v>
+        <v>0.4557</v>
       </c>
       <c r="H26" t="inlineStr"/>
     </row>
@@ -1024,22 +1024,22 @@
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="n">
-        <v>0.2414</v>
+        <v>0.6469</v>
       </c>
       <c r="D27" t="n">
-        <v>0.3402</v>
+        <v>0.595</v>
       </c>
       <c r="E27" t="n">
-        <v>0.231</v>
+        <v>0.4818</v>
       </c>
       <c r="F27" t="n">
-        <v>0.339</v>
+        <v>0.4879</v>
       </c>
       <c r="G27" t="n">
-        <v>0.2087</v>
+        <v>0.5671</v>
       </c>
       <c r="H27" t="n">
-        <v>0.3136</v>
+        <v>0.645</v>
       </c>
     </row>
     <row r="28">
@@ -1050,22 +1050,22 @@
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="n">
-        <v>0.2527</v>
+        <v>0.6772</v>
       </c>
       <c r="D28" t="n">
-        <v>0.2335</v>
+        <v>0.7059</v>
       </c>
       <c r="E28" t="n">
-        <v>0.2088</v>
+        <v>0.4029</v>
       </c>
       <c r="F28" t="n">
-        <v>0.2329</v>
+        <v>0.5236</v>
       </c>
       <c r="G28" t="n">
-        <v>0.2218</v>
+        <v>0.3987</v>
       </c>
       <c r="H28" t="n">
-        <v>0.2058</v>
+        <v>0.2153</v>
       </c>
     </row>
     <row r="29">
@@ -1079,16 +1079,16 @@
         <v>0.2428</v>
       </c>
       <c r="D29" t="n">
-        <v>0.2132</v>
+        <v>0.3451</v>
       </c>
       <c r="E29" t="n">
-        <v>0.2234</v>
+        <v>0.5191</v>
       </c>
       <c r="F29" t="n">
-        <v>0.3606</v>
+        <v>0.554</v>
       </c>
       <c r="G29" t="n">
-        <v>0.3373</v>
+        <v>0.5759</v>
       </c>
       <c r="H29" t="inlineStr"/>
     </row>
@@ -1102,16 +1102,16 @@
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="n">
-        <v>0.2002</v>
+        <v>0.5227000000000001</v>
       </c>
       <c r="F30" t="n">
-        <v>0.2906</v>
+        <v>0.397</v>
       </c>
       <c r="G30" t="n">
-        <v>0.2688</v>
+        <v>0.6692</v>
       </c>
       <c r="H30" t="n">
-        <v>0.2216</v>
+        <v>0.6657999999999999</v>
       </c>
     </row>
     <row r="31">
@@ -1124,13 +1124,13 @@
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="n">
-        <v>0.3054</v>
+        <v>0.5711000000000001</v>
       </c>
       <c r="F31" t="n">
-        <v>0.2661</v>
+        <v>0.5406</v>
       </c>
       <c r="G31" t="n">
-        <v>0.2228</v>
+        <v>0.3878</v>
       </c>
       <c r="H31" t="inlineStr"/>
     </row>
@@ -1142,19 +1142,19 @@
       </c>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="n">
-        <v>0.3086</v>
+        <v>0.3433</v>
       </c>
       <c r="D32" t="n">
-        <v>0.2057</v>
+        <v>0.3453</v>
       </c>
       <c r="E32" t="n">
-        <v>0.2022</v>
+        <v>0.288</v>
       </c>
       <c r="F32" t="n">
-        <v>0.2757</v>
+        <v>0.649</v>
       </c>
       <c r="G32" t="n">
-        <v>0.2601</v>
+        <v>0.3658</v>
       </c>
       <c r="H32" t="inlineStr"/>
     </row>
@@ -1169,13 +1169,13 @@
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr"/>
       <c r="F33" t="n">
-        <v>0.2096</v>
+        <v>0.4726</v>
       </c>
       <c r="G33" t="n">
-        <v>0.2262</v>
+        <v>0.4463</v>
       </c>
       <c r="H33" t="n">
-        <v>0.3332</v>
+        <v>0.4059</v>
       </c>
     </row>
     <row r="34">
@@ -1190,10 +1190,10 @@
       <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="n">
-        <v>0.2218</v>
+        <v>0.4022</v>
       </c>
       <c r="H34" t="n">
-        <v>0.2525</v>
+        <v>0.4597</v>
       </c>
     </row>
     <row r="35">
@@ -1206,16 +1206,16 @@
       <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="n">
-        <v>0.202</v>
+        <v>0.3602</v>
       </c>
       <c r="F35" t="n">
-        <v>0.231</v>
+        <v>0.2942</v>
       </c>
       <c r="G35" t="n">
-        <v>0.2223</v>
+        <v>0.5263</v>
       </c>
       <c r="H35" t="n">
-        <v>0.276</v>
+        <v>0.4855</v>
       </c>
     </row>
     <row r="36">
@@ -1226,19 +1226,19 @@
       </c>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="n">
-        <v>0.3206</v>
+        <v>0.3778</v>
       </c>
       <c r="D36" t="n">
-        <v>0.3949</v>
+        <v>0.5175</v>
       </c>
       <c r="E36" t="n">
-        <v>0.272</v>
+        <v>0.4899</v>
       </c>
       <c r="F36" t="n">
-        <v>0.2241</v>
+        <v>0.2545</v>
       </c>
       <c r="G36" t="n">
-        <v>0.2105</v>
+        <v>0.6035</v>
       </c>
       <c r="H36" t="inlineStr"/>
     </row>
@@ -1251,10 +1251,10 @@
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="n">
-        <v>0.286</v>
+        <v>0.418</v>
       </c>
       <c r="E37" t="n">
-        <v>0.2022</v>
+        <v>0.4288</v>
       </c>
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="n">
@@ -1270,7 +1270,7 @@
       </c>
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="n">
-        <v>0.3572</v>
+        <v>0.6499</v>
       </c>
       <c r="D38" t="n">
         <v>0.6555</v>
@@ -1279,10 +1279,10 @@
         <v>0.3854</v>
       </c>
       <c r="F38" t="n">
-        <v>0.2212</v>
+        <v>0.3375</v>
       </c>
       <c r="G38" t="n">
-        <v>0.2787</v>
+        <v>0.7084</v>
       </c>
       <c r="H38" t="inlineStr"/>
     </row>
@@ -1297,10 +1297,10 @@
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr"/>
       <c r="F39" t="n">
-        <v>0.2105</v>
+        <v>0.4438</v>
       </c>
       <c r="G39" t="n">
-        <v>0.237</v>
+        <v>0.5869</v>
       </c>
       <c r="H39" t="inlineStr"/>
     </row>
@@ -1315,13 +1315,13 @@
         <v>0.3886</v>
       </c>
       <c r="D40" t="n">
-        <v>0.2553</v>
+        <v>0.3933</v>
       </c>
       <c r="E40" t="n">
-        <v>0.203</v>
+        <v>0.2271</v>
       </c>
       <c r="F40" t="n">
-        <v>0.2276</v>
+        <v>0.3753</v>
       </c>
       <c r="G40" t="n">
         <v>0.2336</v>
@@ -1336,7 +1336,7 @@
       </c>
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="n">
-        <v>0.2283</v>
+        <v>0.2332</v>
       </c>
       <c r="D41" t="n">
         <v>0.2021</v>
@@ -1345,10 +1345,10 @@
         <v>0.2097</v>
       </c>
       <c r="F41" t="n">
-        <v>0.2225</v>
+        <v>0.323</v>
       </c>
       <c r="G41" t="n">
-        <v>0.2195</v>
+        <v>0.2242</v>
       </c>
       <c r="H41" t="inlineStr"/>
     </row>
@@ -1360,19 +1360,19 @@
       </c>
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="n">
-        <v>0.2617</v>
+        <v>0.3956</v>
       </c>
       <c r="D42" t="n">
-        <v>0.2815</v>
+        <v>0.3753</v>
       </c>
       <c r="E42" t="n">
-        <v>0.2089</v>
+        <v>0.5266</v>
       </c>
       <c r="F42" t="n">
-        <v>0.2167</v>
+        <v>0.4266</v>
       </c>
       <c r="G42" t="n">
-        <v>0.2154</v>
+        <v>0.4145</v>
       </c>
       <c r="H42" t="inlineStr"/>
     </row>
@@ -1384,22 +1384,22 @@
       </c>
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="n">
-        <v>0.2956</v>
+        <v>0.3783</v>
       </c>
       <c r="D43" t="n">
-        <v>0.2305</v>
+        <v>0.4807</v>
       </c>
       <c r="E43" t="n">
-        <v>0.2113</v>
+        <v>0.27</v>
       </c>
       <c r="F43" t="n">
-        <v>0.2922</v>
+        <v>0.575</v>
       </c>
       <c r="G43" t="n">
-        <v>0.2091</v>
+        <v>0.3515</v>
       </c>
       <c r="H43" t="n">
-        <v>0.2456</v>
+        <v>0.3518</v>
       </c>
     </row>
     <row r="44">
@@ -1413,13 +1413,13 @@
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr"/>
       <c r="F44" t="n">
-        <v>0.3476</v>
+        <v>0.3872</v>
       </c>
       <c r="G44" t="n">
-        <v>0.3048</v>
+        <v>0.4144</v>
       </c>
       <c r="H44" t="n">
-        <v>0.2035</v>
+        <v>0.5336</v>
       </c>
     </row>
     <row r="45">
@@ -1431,13 +1431,13 @@
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="n">
-        <v>0.2701</v>
+        <v>0.3962</v>
       </c>
       <c r="E45" t="n">
         <v>0.253</v>
       </c>
       <c r="F45" t="n">
-        <v>0.2404</v>
+        <v>0.3359</v>
       </c>
       <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr"/>
@@ -1451,16 +1451,16 @@
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr"/>
       <c r="D46" t="n">
-        <v>0.2073</v>
+        <v>0.2955</v>
       </c>
       <c r="E46" t="n">
-        <v>0.2225</v>
+        <v>0.4465</v>
       </c>
       <c r="F46" t="n">
-        <v>0.237</v>
+        <v>0.3243</v>
       </c>
       <c r="G46" t="n">
-        <v>0.2223</v>
+        <v>0.2475</v>
       </c>
       <c r="H46" t="n">
         <v>0.3382</v>
@@ -1474,19 +1474,19 @@
       </c>
       <c r="B47" t="inlineStr"/>
       <c r="C47" t="n">
-        <v>0.2018</v>
+        <v>0.3494</v>
       </c>
       <c r="D47" t="n">
-        <v>0.2951</v>
+        <v>0.5231</v>
       </c>
       <c r="E47" t="n">
-        <v>0.2067</v>
+        <v>0.32</v>
       </c>
       <c r="F47" t="n">
-        <v>0.2169</v>
+        <v>0.3277</v>
       </c>
       <c r="G47" t="n">
-        <v>0.201</v>
+        <v>0.3437</v>
       </c>
       <c r="H47" t="inlineStr"/>
     </row>
@@ -1503,10 +1503,10 @@
         <v>0.362</v>
       </c>
       <c r="F48" t="n">
-        <v>0.2148</v>
+        <v>0.2931</v>
       </c>
       <c r="G48" t="n">
-        <v>0.2038</v>
+        <v>0.2287</v>
       </c>
       <c r="H48" t="inlineStr"/>
     </row>
@@ -1518,19 +1518,19 @@
       </c>
       <c r="B49" t="inlineStr"/>
       <c r="C49" t="n">
-        <v>0.2222</v>
+        <v>0.4815</v>
       </c>
       <c r="D49" t="n">
-        <v>0.2132</v>
+        <v>0.3422</v>
       </c>
       <c r="E49" t="n">
-        <v>0.2176</v>
+        <v>0.4552</v>
       </c>
       <c r="F49" t="n">
-        <v>0.2051</v>
+        <v>0.3364</v>
       </c>
       <c r="G49" t="n">
-        <v>0.2182</v>
+        <v>0.3983</v>
       </c>
       <c r="H49" t="inlineStr"/>
     </row>
@@ -1544,13 +1544,13 @@
       <c r="C50" t="inlineStr"/>
       <c r="D50" t="inlineStr"/>
       <c r="E50" t="n">
-        <v>0.2945</v>
+        <v>0.4601</v>
       </c>
       <c r="F50" t="n">
-        <v>0.2764</v>
+        <v>0.4151</v>
       </c>
       <c r="G50" t="n">
-        <v>0.2391</v>
+        <v>0.3985</v>
       </c>
       <c r="H50" t="n">
         <v>0.4229</v>
@@ -1565,19 +1565,19 @@
       <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr"/>
       <c r="D51" t="n">
-        <v>0.2987</v>
+        <v>0.3101</v>
       </c>
       <c r="E51" t="n">
-        <v>0.2061</v>
+        <v>0.2191</v>
       </c>
       <c r="F51" t="n">
-        <v>0.3875</v>
+        <v>0.4091</v>
       </c>
       <c r="G51" t="n">
-        <v>0.2559</v>
+        <v>0.2681</v>
       </c>
       <c r="H51" t="n">
-        <v>0.3011</v>
+        <v>0.3715</v>
       </c>
     </row>
     <row r="52">
@@ -1588,19 +1588,19 @@
       </c>
       <c r="B52" t="inlineStr"/>
       <c r="C52" t="n">
-        <v>0.3022</v>
+        <v>0.4315</v>
       </c>
       <c r="D52" t="n">
         <v>0.2023</v>
       </c>
       <c r="E52" t="n">
-        <v>0.2054</v>
+        <v>0.2868</v>
       </c>
       <c r="F52" t="n">
         <v>0.2926</v>
       </c>
       <c r="G52" t="n">
-        <v>0.2153</v>
+        <v>0.3105</v>
       </c>
       <c r="H52" t="inlineStr"/>
     </row>
@@ -1612,19 +1612,19 @@
       </c>
       <c r="B53" t="inlineStr"/>
       <c r="C53" t="n">
-        <v>0.3033</v>
+        <v>0.3494</v>
       </c>
       <c r="D53" t="n">
-        <v>0.2537</v>
+        <v>0.3039</v>
       </c>
       <c r="E53" t="n">
-        <v>0.256</v>
+        <v>0.2724</v>
       </c>
       <c r="F53" t="n">
-        <v>0.2376</v>
+        <v>0.2779</v>
       </c>
       <c r="G53" t="n">
-        <v>0.3574</v>
+        <v>0.3646</v>
       </c>
       <c r="H53" t="inlineStr"/>
     </row>
@@ -1636,16 +1636,16 @@
       </c>
       <c r="B54" t="inlineStr"/>
       <c r="C54" t="n">
-        <v>0.2082</v>
+        <v>0.3943</v>
       </c>
       <c r="D54" t="n">
-        <v>0.2315</v>
+        <v>0.3356</v>
       </c>
       <c r="E54" t="n">
-        <v>0.2917</v>
+        <v>0.4832</v>
       </c>
       <c r="F54" t="n">
-        <v>0.3343</v>
+        <v>0.3808</v>
       </c>
       <c r="G54" t="n">
         <v>0.4699</v>
@@ -1660,19 +1660,19 @@
       </c>
       <c r="B55" t="inlineStr"/>
       <c r="C55" t="n">
-        <v>0.3559</v>
+        <v>0.6892</v>
       </c>
       <c r="D55" t="n">
-        <v>0.2186</v>
+        <v>0.2487</v>
       </c>
       <c r="E55" t="n">
-        <v>0.2094</v>
+        <v>0.2889</v>
       </c>
       <c r="F55" t="n">
-        <v>0.2512</v>
+        <v>0.4984</v>
       </c>
       <c r="G55" t="n">
-        <v>0.2639</v>
+        <v>0.2677</v>
       </c>
       <c r="H55" t="inlineStr"/>
     </row>
@@ -1687,16 +1687,16 @@
         <v>0.2079</v>
       </c>
       <c r="D56" t="n">
-        <v>0.2817</v>
+        <v>0.3362</v>
       </c>
       <c r="E56" t="n">
-        <v>0.2257</v>
+        <v>0.3241</v>
       </c>
       <c r="F56" t="n">
-        <v>0.2239</v>
+        <v>0.2438</v>
       </c>
       <c r="G56" t="n">
-        <v>0.2107</v>
+        <v>0.2457</v>
       </c>
       <c r="H56" t="inlineStr"/>
     </row>
@@ -1708,19 +1708,19 @@
       </c>
       <c r="B57" t="inlineStr"/>
       <c r="C57" t="n">
-        <v>0.2896</v>
+        <v>0.5215</v>
       </c>
       <c r="D57" t="n">
-        <v>0.2907</v>
+        <v>0.5873</v>
       </c>
       <c r="E57" t="n">
-        <v>0.3141</v>
+        <v>0.5377</v>
       </c>
       <c r="F57" t="n">
-        <v>0.2175</v>
+        <v>0.4444</v>
       </c>
       <c r="G57" t="n">
-        <v>0.2402</v>
+        <v>0.5313</v>
       </c>
       <c r="H57" t="inlineStr"/>
     </row>
@@ -1732,19 +1732,19 @@
       </c>
       <c r="B58" t="inlineStr"/>
       <c r="C58" t="n">
-        <v>0.2017</v>
+        <v>0.5673</v>
       </c>
       <c r="D58" t="n">
-        <v>0.2466</v>
+        <v>0.4516</v>
       </c>
       <c r="E58" t="n">
-        <v>0.2885</v>
+        <v>0.3962</v>
       </c>
       <c r="F58" t="n">
-        <v>0.231</v>
+        <v>0.3732</v>
       </c>
       <c r="G58" t="n">
-        <v>0.2157</v>
+        <v>0.4301</v>
       </c>
       <c r="H58" t="inlineStr"/>
     </row>
@@ -1755,22 +1755,22 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>0.2129</v>
+        <v>0.3825</v>
       </c>
       <c r="C59" t="n">
-        <v>0.2136</v>
+        <v>0.3607</v>
       </c>
       <c r="D59" t="n">
-        <v>0.2187</v>
+        <v>0.3887</v>
       </c>
       <c r="E59" t="n">
-        <v>0.2281</v>
+        <v>0.5352</v>
       </c>
       <c r="F59" t="n">
-        <v>0.3277</v>
+        <v>0.4762</v>
       </c>
       <c r="G59" t="n">
-        <v>0.2432</v>
+        <v>0.3254</v>
       </c>
       <c r="H59" t="inlineStr"/>
     </row>
@@ -1781,22 +1781,22 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>0.248</v>
+        <v>0.4277</v>
       </c>
       <c r="C60" t="n">
-        <v>0.2618</v>
+        <v>0.4903</v>
       </c>
       <c r="D60" t="n">
-        <v>0.2358</v>
+        <v>0.5182</v>
       </c>
       <c r="E60" t="n">
-        <v>0.2138</v>
+        <v>0.4458</v>
       </c>
       <c r="F60" t="n">
-        <v>0.2229</v>
+        <v>0.4116</v>
       </c>
       <c r="G60" t="n">
-        <v>0.2092</v>
+        <v>0.2747</v>
       </c>
       <c r="H60" t="inlineStr"/>
     </row>
@@ -1807,22 +1807,22 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>0.2114</v>
+        <v>0.3571</v>
       </c>
       <c r="C61" t="n">
-        <v>0.225</v>
+        <v>0.408</v>
       </c>
       <c r="D61" t="n">
-        <v>0.2864</v>
+        <v>0.4338</v>
       </c>
       <c r="E61" t="n">
-        <v>0.2541</v>
+        <v>0.3295</v>
       </c>
       <c r="F61" t="n">
-        <v>0.2403</v>
+        <v>0.4508</v>
       </c>
       <c r="G61" t="n">
-        <v>0.2309</v>
+        <v>0.3527</v>
       </c>
       <c r="H61" t="inlineStr"/>
     </row>
@@ -1840,10 +1840,10 @@
         <v>0.2576</v>
       </c>
       <c r="E62" t="n">
-        <v>0.2234</v>
+        <v>0.2755</v>
       </c>
       <c r="F62" t="n">
-        <v>0.2788</v>
+        <v>0.451</v>
       </c>
       <c r="G62" t="n">
         <v>0.326</v>
@@ -1858,16 +1858,16 @@
       </c>
       <c r="B63" t="inlineStr"/>
       <c r="C63" t="n">
-        <v>0.2246</v>
+        <v>0.25</v>
       </c>
       <c r="D63" t="n">
-        <v>0.2113</v>
+        <v>0.2592</v>
       </c>
       <c r="E63" t="n">
-        <v>0.2053</v>
+        <v>0.2598</v>
       </c>
       <c r="F63" t="n">
-        <v>0.2857</v>
+        <v>0.4195</v>
       </c>
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr"/>
@@ -1880,19 +1880,19 @@
       </c>
       <c r="B64" t="inlineStr"/>
       <c r="C64" t="n">
-        <v>0.2476</v>
+        <v>0.4799</v>
       </c>
       <c r="D64" t="n">
-        <v>0.2644</v>
+        <v>0.3662</v>
       </c>
       <c r="E64" t="n">
-        <v>0.5169</v>
+        <v>0.6795</v>
       </c>
       <c r="F64" t="n">
-        <v>0.4755</v>
+        <v>0.6607</v>
       </c>
       <c r="G64" t="n">
-        <v>0.2839</v>
+        <v>0.7028</v>
       </c>
       <c r="H64" t="inlineStr"/>
     </row>
@@ -1906,13 +1906,13 @@
       <c r="C65" t="inlineStr"/>
       <c r="D65" t="inlineStr"/>
       <c r="E65" t="n">
-        <v>0.3053</v>
+        <v>0.6157</v>
       </c>
       <c r="F65" t="n">
-        <v>0.2373</v>
+        <v>0.5925</v>
       </c>
       <c r="G65" t="n">
-        <v>0.4062</v>
+        <v>0.6972</v>
       </c>
       <c r="H65" t="inlineStr"/>
     </row>
@@ -1924,19 +1924,19 @@
       </c>
       <c r="B66" t="inlineStr"/>
       <c r="C66" t="n">
-        <v>0.2199</v>
+        <v>0.5463</v>
       </c>
       <c r="D66" t="n">
-        <v>0.2399</v>
+        <v>0.4723</v>
       </c>
       <c r="E66" t="n">
-        <v>0.2111</v>
+        <v>0.4369</v>
       </c>
       <c r="F66" t="n">
-        <v>0.2837</v>
+        <v>0.3025</v>
       </c>
       <c r="G66" t="n">
-        <v>0.217</v>
+        <v>0.287</v>
       </c>
       <c r="H66" t="inlineStr"/>
     </row>
@@ -1948,19 +1948,19 @@
       </c>
       <c r="B67" t="inlineStr"/>
       <c r="C67" t="n">
-        <v>0.3126</v>
+        <v>0.3608</v>
       </c>
       <c r="D67" t="n">
-        <v>0.3262</v>
+        <v>0.3498</v>
       </c>
       <c r="E67" t="n">
         <v>0.3728</v>
       </c>
       <c r="F67" t="n">
-        <v>0.2238</v>
+        <v>0.4195</v>
       </c>
       <c r="G67" t="n">
-        <v>0.3065</v>
+        <v>0.34</v>
       </c>
       <c r="H67" t="inlineStr"/>
     </row>
@@ -1972,19 +1972,19 @@
       </c>
       <c r="B68" t="inlineStr"/>
       <c r="C68" t="n">
-        <v>0.2512</v>
+        <v>0.6282</v>
       </c>
       <c r="D68" t="n">
-        <v>0.2748</v>
+        <v>0.6111</v>
       </c>
       <c r="E68" t="n">
-        <v>0.2404</v>
+        <v>0.5292</v>
       </c>
       <c r="F68" t="n">
-        <v>0.2137</v>
+        <v>0.4627</v>
       </c>
       <c r="G68" t="n">
-        <v>0.2361</v>
+        <v>0.5214</v>
       </c>
       <c r="H68" t="inlineStr"/>
     </row>
@@ -1996,16 +1996,16 @@
       </c>
       <c r="B69" t="inlineStr"/>
       <c r="C69" t="n">
-        <v>0.2085</v>
+        <v>0.3701</v>
       </c>
       <c r="D69" t="n">
-        <v>0.2162</v>
+        <v>0.4725</v>
       </c>
       <c r="E69" t="n">
-        <v>0.335</v>
+        <v>0.5617</v>
       </c>
       <c r="F69" t="n">
-        <v>0.2128</v>
+        <v>0.4239</v>
       </c>
       <c r="G69" t="inlineStr"/>
       <c r="H69" t="inlineStr"/>
@@ -2018,16 +2018,16 @@
       </c>
       <c r="B70" t="inlineStr"/>
       <c r="C70" t="n">
-        <v>0.2284</v>
+        <v>0.3474</v>
       </c>
       <c r="D70" t="n">
-        <v>0.2498</v>
+        <v>0.3276</v>
       </c>
       <c r="E70" t="n">
-        <v>0.223</v>
+        <v>0.2477</v>
       </c>
       <c r="F70" t="n">
-        <v>0.2233</v>
+        <v>0.2978</v>
       </c>
       <c r="G70" t="inlineStr"/>
       <c r="H70" t="inlineStr"/>
@@ -2040,22 +2040,22 @@
       </c>
       <c r="B71" t="inlineStr"/>
       <c r="C71" t="n">
-        <v>0.2787</v>
+        <v>0.356</v>
       </c>
       <c r="D71" t="n">
-        <v>0.2199</v>
+        <v>0.3777</v>
       </c>
       <c r="E71" t="n">
-        <v>0.2302</v>
+        <v>0.3285</v>
       </c>
       <c r="F71" t="n">
-        <v>0.2508</v>
+        <v>0.313</v>
       </c>
       <c r="G71" t="n">
-        <v>0.2535</v>
+        <v>0.3941</v>
       </c>
       <c r="H71" t="n">
-        <v>0.2943</v>
+        <v>0.3004</v>
       </c>
     </row>
     <row r="72">
@@ -2066,19 +2066,19 @@
       </c>
       <c r="B72" t="inlineStr"/>
       <c r="C72" t="n">
-        <v>0.2876</v>
+        <v>0.3928</v>
       </c>
       <c r="D72" t="n">
-        <v>0.2962</v>
+        <v>0.3851</v>
       </c>
       <c r="E72" t="n">
-        <v>0.2352</v>
+        <v>0.3275</v>
       </c>
       <c r="F72" t="n">
-        <v>0.2169</v>
+        <v>0.3955</v>
       </c>
       <c r="G72" t="n">
-        <v>0.2642</v>
+        <v>0.3498</v>
       </c>
       <c r="H72" t="inlineStr"/>
     </row>
@@ -2090,19 +2090,19 @@
       </c>
       <c r="B73" t="inlineStr"/>
       <c r="C73" t="n">
-        <v>0.27</v>
+        <v>0.309</v>
       </c>
       <c r="D73" t="n">
-        <v>0.2185</v>
+        <v>0.2791</v>
       </c>
       <c r="E73" t="n">
-        <v>0.234</v>
+        <v>0.3329</v>
       </c>
       <c r="F73" t="n">
-        <v>0.2898</v>
+        <v>0.5734</v>
       </c>
       <c r="G73" t="n">
-        <v>0.2659</v>
+        <v>0.3006</v>
       </c>
       <c r="H73" t="inlineStr"/>
     </row>
@@ -2114,16 +2114,16 @@
       </c>
       <c r="B74" t="inlineStr"/>
       <c r="C74" t="n">
-        <v>0.2284</v>
+        <v>0.3678</v>
       </c>
       <c r="D74" t="n">
-        <v>0.2303</v>
+        <v>0.2393</v>
       </c>
       <c r="E74" t="n">
-        <v>0.2813</v>
+        <v>0.3259</v>
       </c>
       <c r="F74" t="n">
-        <v>0.219</v>
+        <v>0.4245</v>
       </c>
       <c r="G74" t="inlineStr"/>
       <c r="H74" t="inlineStr"/>
@@ -2136,19 +2136,19 @@
       </c>
       <c r="B75" t="inlineStr"/>
       <c r="C75" t="n">
-        <v>0.2429</v>
+        <v>0.5748</v>
       </c>
       <c r="D75" t="n">
-        <v>0.2514</v>
+        <v>0.4787</v>
       </c>
       <c r="E75" t="n">
-        <v>0.2157</v>
+        <v>0.5348000000000001</v>
       </c>
       <c r="F75" t="n">
-        <v>0.2111</v>
+        <v>0.3941</v>
       </c>
       <c r="G75" t="n">
-        <v>0.2156</v>
+        <v>0.4488</v>
       </c>
       <c r="H75" t="inlineStr"/>
     </row>
@@ -2160,16 +2160,16 @@
       </c>
       <c r="B76" t="inlineStr"/>
       <c r="C76" t="n">
-        <v>0.2382</v>
+        <v>0.3121</v>
       </c>
       <c r="D76" t="n">
-        <v>0.3037</v>
+        <v>0.5291</v>
       </c>
       <c r="E76" t="n">
-        <v>0.222</v>
+        <v>0.2571</v>
       </c>
       <c r="F76" t="n">
-        <v>0.2181</v>
+        <v>0.2791</v>
       </c>
       <c r="G76" t="inlineStr"/>
       <c r="H76" t="inlineStr"/>
@@ -2182,16 +2182,16 @@
       </c>
       <c r="B77" t="inlineStr"/>
       <c r="C77" t="n">
-        <v>0.2084</v>
+        <v>0.3078</v>
       </c>
       <c r="D77" t="n">
-        <v>0.2541</v>
+        <v>0.263</v>
       </c>
       <c r="E77" t="n">
-        <v>0.2019</v>
+        <v>0.4606</v>
       </c>
       <c r="F77" t="n">
-        <v>0.2484</v>
+        <v>0.4836</v>
       </c>
       <c r="G77" t="n">
         <v>0.226</v>
@@ -2206,19 +2206,19 @@
       </c>
       <c r="B78" t="inlineStr"/>
       <c r="C78" t="n">
-        <v>0.2394</v>
+        <v>0.3539</v>
       </c>
       <c r="D78" t="n">
-        <v>0.2001</v>
+        <v>0.2757</v>
       </c>
       <c r="E78" t="n">
         <v>0.2079</v>
       </c>
       <c r="F78" t="n">
-        <v>0.2028</v>
+        <v>0.2372</v>
       </c>
       <c r="G78" t="n">
-        <v>0.2313</v>
+        <v>0.5838</v>
       </c>
       <c r="H78" t="inlineStr"/>
     </row>
@@ -2233,16 +2233,16 @@
         <v>0.3486</v>
       </c>
       <c r="D79" t="n">
-        <v>0.2484</v>
+        <v>0.2727</v>
       </c>
       <c r="E79" t="n">
-        <v>0.2086</v>
+        <v>0.4444</v>
       </c>
       <c r="F79" t="n">
-        <v>0.3601</v>
+        <v>0.3954</v>
       </c>
       <c r="G79" t="n">
-        <v>0.3945</v>
+        <v>0.446</v>
       </c>
       <c r="H79" t="inlineStr"/>
     </row>
@@ -2263,7 +2263,7 @@
         <v>0.349</v>
       </c>
       <c r="F80" t="n">
-        <v>0.2562</v>
+        <v>0.3913</v>
       </c>
       <c r="G80" t="inlineStr"/>
       <c r="H80" t="inlineStr"/>
@@ -2276,19 +2276,19 @@
       </c>
       <c r="B81" t="inlineStr"/>
       <c r="C81" t="n">
-        <v>0.268</v>
+        <v>0.348</v>
       </c>
       <c r="D81" t="n">
-        <v>0.2435</v>
+        <v>0.3622</v>
       </c>
       <c r="E81" t="n">
-        <v>0.252</v>
+        <v>0.3641</v>
       </c>
       <c r="F81" t="n">
-        <v>0.2354</v>
+        <v>0.3075</v>
       </c>
       <c r="G81" t="n">
-        <v>0.3136</v>
+        <v>0.3475</v>
       </c>
       <c r="H81" t="inlineStr"/>
     </row>
@@ -2300,19 +2300,19 @@
       </c>
       <c r="B82" t="inlineStr"/>
       <c r="C82" t="n">
-        <v>0.2268</v>
+        <v>0.4722</v>
       </c>
       <c r="D82" t="n">
-        <v>0.2082</v>
+        <v>0.3044</v>
       </c>
       <c r="E82" t="n">
-        <v>0.2593</v>
+        <v>0.3951</v>
       </c>
       <c r="F82" t="n">
-        <v>0.2461</v>
+        <v>0.4123</v>
       </c>
       <c r="G82" t="n">
-        <v>0.2717</v>
+        <v>0.2827</v>
       </c>
       <c r="H82" t="inlineStr"/>
     </row>
@@ -2323,19 +2323,19 @@
         </is>
       </c>
       <c r="B83" t="n">
-        <v>0.2013</v>
+        <v>0.3605</v>
       </c>
       <c r="C83" t="n">
-        <v>0.3669</v>
+        <v>0.7184</v>
       </c>
       <c r="D83" t="n">
-        <v>0.3452</v>
+        <v>0.523</v>
       </c>
       <c r="E83" t="n">
-        <v>0.4628</v>
+        <v>0.7012</v>
       </c>
       <c r="F83" t="n">
-        <v>0.4298</v>
+        <v>0.5685</v>
       </c>
       <c r="G83" t="inlineStr"/>
       <c r="H83" t="inlineStr"/>
@@ -2347,22 +2347,22 @@
         </is>
       </c>
       <c r="B84" t="n">
-        <v>0.3206</v>
+        <v>0.6031</v>
       </c>
       <c r="C84" t="n">
-        <v>0.2372</v>
+        <v>0.4726</v>
       </c>
       <c r="D84" t="n">
-        <v>0.2639</v>
+        <v>0.5044</v>
       </c>
       <c r="E84" t="n">
-        <v>0.2732</v>
+        <v>0.5723</v>
       </c>
       <c r="F84" t="n">
-        <v>0.3104</v>
+        <v>0.4545</v>
       </c>
       <c r="G84" t="n">
-        <v>0.2171</v>
+        <v>0.5108</v>
       </c>
       <c r="H84" t="inlineStr"/>
     </row>
@@ -2374,19 +2374,19 @@
       </c>
       <c r="B85" t="inlineStr"/>
       <c r="C85" t="n">
-        <v>0.2323</v>
+        <v>0.374</v>
       </c>
       <c r="D85" t="n">
-        <v>0.3511</v>
+        <v>0.391</v>
       </c>
       <c r="E85" t="n">
-        <v>0.2321</v>
+        <v>0.316</v>
       </c>
       <c r="F85" t="n">
-        <v>0.2846</v>
+        <v>0.6362</v>
       </c>
       <c r="G85" t="n">
-        <v>0.2196</v>
+        <v>0.388</v>
       </c>
       <c r="H85" t="inlineStr"/>
     </row>
@@ -2397,10 +2397,10 @@
         </is>
       </c>
       <c r="B86" t="n">
-        <v>0.5449000000000001</v>
+        <v>0.6662</v>
       </c>
       <c r="C86" t="n">
-        <v>0.3687</v>
+        <v>0.4327</v>
       </c>
       <c r="D86" t="n">
         <v>0.4118</v>
@@ -2427,7 +2427,7 @@
         <v>0.2171</v>
       </c>
       <c r="F87" t="n">
-        <v>0.2825</v>
+        <v>0.3488</v>
       </c>
       <c r="G87" t="inlineStr"/>
       <c r="H87" t="inlineStr"/>
@@ -2442,16 +2442,16 @@
       <c r="C88" t="inlineStr"/>
       <c r="D88" t="inlineStr"/>
       <c r="E88" t="n">
-        <v>0.2286</v>
+        <v>0.3062</v>
       </c>
       <c r="F88" t="n">
-        <v>0.229</v>
+        <v>0.3096</v>
       </c>
       <c r="G88" t="n">
-        <v>0.3149</v>
+        <v>0.3725</v>
       </c>
       <c r="H88" t="n">
-        <v>0.3149</v>
+        <v>0.3725</v>
       </c>
     </row>
     <row r="89">
@@ -2464,16 +2464,16 @@
       <c r="C89" t="inlineStr"/>
       <c r="D89" t="inlineStr"/>
       <c r="E89" t="n">
-        <v>0.2057</v>
+        <v>0.583</v>
       </c>
       <c r="F89" t="n">
-        <v>0.3199</v>
+        <v>0.5465</v>
       </c>
       <c r="G89" t="n">
-        <v>0.2298</v>
+        <v>0.6515</v>
       </c>
       <c r="H89" t="n">
-        <v>0.2223</v>
+        <v>0.6368</v>
       </c>
     </row>
     <row r="90">
@@ -2487,13 +2487,13 @@
       <c r="D90" t="inlineStr"/>
       <c r="E90" t="inlineStr"/>
       <c r="F90" t="n">
-        <v>0.2857</v>
+        <v>0.4496</v>
       </c>
       <c r="G90" t="n">
-        <v>0.22</v>
+        <v>0.4069</v>
       </c>
       <c r="H90" t="n">
-        <v>0.2037</v>
+        <v>0.4441</v>
       </c>
     </row>
     <row r="91">
@@ -2504,16 +2504,16 @@
       </c>
       <c r="B91" t="inlineStr"/>
       <c r="C91" t="n">
-        <v>0.2228</v>
+        <v>0.4649</v>
       </c>
       <c r="D91" t="n">
-        <v>0.3902</v>
+        <v>0.6209</v>
       </c>
       <c r="E91" t="n">
-        <v>0.3096</v>
+        <v>0.5846</v>
       </c>
       <c r="F91" t="n">
-        <v>0.21</v>
+        <v>0.4347</v>
       </c>
       <c r="G91" t="inlineStr"/>
       <c r="H91" t="inlineStr"/>
@@ -2525,19 +2525,19 @@
         </is>
       </c>
       <c r="B92" t="n">
-        <v>0.3543</v>
+        <v>0.4114</v>
       </c>
       <c r="C92" t="n">
-        <v>0.2809</v>
+        <v>0.3246</v>
       </c>
       <c r="D92" t="n">
-        <v>0.2061</v>
+        <v>0.3222</v>
       </c>
       <c r="E92" t="n">
-        <v>0.2698</v>
+        <v>0.403</v>
       </c>
       <c r="F92" t="n">
-        <v>0.21</v>
+        <v>0.3458</v>
       </c>
       <c r="G92" t="inlineStr"/>
       <c r="H92" t="inlineStr"/>
@@ -2550,16 +2550,16 @@
       </c>
       <c r="B93" t="inlineStr"/>
       <c r="C93" t="n">
-        <v>0.2129</v>
+        <v>0.5125999999999999</v>
       </c>
       <c r="D93" t="n">
-        <v>0.2411</v>
+        <v>0.4346</v>
       </c>
       <c r="E93" t="n">
-        <v>0.2678</v>
+        <v>0.4698</v>
       </c>
       <c r="F93" t="n">
-        <v>0.2251</v>
+        <v>0.4343</v>
       </c>
       <c r="G93" t="inlineStr"/>
       <c r="H93" t="inlineStr"/>
@@ -2571,19 +2571,19 @@
         </is>
       </c>
       <c r="B94" t="n">
-        <v>0.2233</v>
+        <v>0.4526</v>
       </c>
       <c r="C94" t="n">
-        <v>0.2022</v>
+        <v>0.2946</v>
       </c>
       <c r="D94" t="n">
-        <v>0.2414</v>
+        <v>0.4498</v>
       </c>
       <c r="E94" t="n">
-        <v>0.2239</v>
+        <v>0.3451</v>
       </c>
       <c r="F94" t="n">
-        <v>0.2126</v>
+        <v>0.4156</v>
       </c>
       <c r="G94" t="inlineStr"/>
       <c r="H94" t="inlineStr"/>
@@ -2595,19 +2595,19 @@
         </is>
       </c>
       <c r="B95" t="n">
-        <v>0.2022</v>
+        <v>0.4777</v>
       </c>
       <c r="C95" t="n">
-        <v>0.3556</v>
+        <v>0.5196</v>
       </c>
       <c r="D95" t="n">
-        <v>0.2138</v>
+        <v>0.4249</v>
       </c>
       <c r="E95" t="n">
-        <v>0.2243</v>
+        <v>0.3815</v>
       </c>
       <c r="F95" t="n">
-        <v>0.2064</v>
+        <v>0.394</v>
       </c>
       <c r="G95" t="inlineStr"/>
       <c r="H95" t="inlineStr"/>
@@ -2620,19 +2620,19 @@
       </c>
       <c r="B96" t="inlineStr"/>
       <c r="C96" t="n">
-        <v>0.283</v>
+        <v>0.5954</v>
       </c>
       <c r="D96" t="n">
-        <v>0.2657</v>
+        <v>0.5591</v>
       </c>
       <c r="E96" t="n">
-        <v>0.2408</v>
+        <v>0.5017</v>
       </c>
       <c r="F96" t="n">
-        <v>0.2298</v>
+        <v>0.4029</v>
       </c>
       <c r="G96" t="n">
-        <v>0.2612</v>
+        <v>0.489</v>
       </c>
       <c r="H96" t="inlineStr"/>
     </row>
@@ -2644,19 +2644,19 @@
       </c>
       <c r="B97" t="inlineStr"/>
       <c r="C97" t="n">
-        <v>0.2008</v>
+        <v>0.5204</v>
       </c>
       <c r="D97" t="n">
-        <v>0.206</v>
+        <v>0.4495</v>
       </c>
       <c r="E97" t="n">
-        <v>0.2283</v>
+        <v>0.4228</v>
       </c>
       <c r="F97" t="n">
-        <v>0.2133</v>
+        <v>0.533</v>
       </c>
       <c r="G97" t="n">
-        <v>0.2114</v>
+        <v>0.4649</v>
       </c>
       <c r="H97" t="inlineStr"/>
     </row>
@@ -2671,14 +2671,14 @@
         <v>0.2349</v>
       </c>
       <c r="D98" t="n">
-        <v>0.295</v>
+        <v>0.5774</v>
       </c>
       <c r="E98" t="n">
-        <v>0.2151</v>
+        <v>0.5308</v>
       </c>
       <c r="F98" t="inlineStr"/>
       <c r="G98" t="n">
-        <v>0.3119</v>
+        <v>0.6402</v>
       </c>
       <c r="H98" t="inlineStr"/>
     </row>
@@ -2690,19 +2690,19 @@
       </c>
       <c r="B99" t="inlineStr"/>
       <c r="C99" t="n">
-        <v>0.2565</v>
+        <v>0.6758999999999999</v>
       </c>
       <c r="D99" t="n">
-        <v>0.4071</v>
+        <v>0.5239</v>
       </c>
       <c r="E99" t="n">
-        <v>0.332</v>
+        <v>0.6816</v>
       </c>
       <c r="F99" t="n">
-        <v>0.2479</v>
+        <v>0.6563</v>
       </c>
       <c r="G99" t="n">
-        <v>0.2479</v>
+        <v>0.6221</v>
       </c>
       <c r="H99" t="inlineStr"/>
     </row>
@@ -2714,19 +2714,19 @@
       </c>
       <c r="B100" t="inlineStr"/>
       <c r="C100" t="n">
-        <v>0.2138</v>
+        <v>0.6341</v>
       </c>
       <c r="D100" t="n">
         <v>0.4148</v>
       </c>
       <c r="E100" t="n">
-        <v>0.3048</v>
+        <v>0.5221</v>
       </c>
       <c r="F100" t="n">
-        <v>0.2152</v>
+        <v>0.5241</v>
       </c>
       <c r="G100" t="n">
-        <v>0.2575</v>
+        <v>0.467</v>
       </c>
       <c r="H100" t="inlineStr"/>
     </row>
@@ -2738,22 +2738,22 @@
       </c>
       <c r="B101" t="inlineStr"/>
       <c r="C101" t="n">
-        <v>0.2162</v>
+        <v>0.4635</v>
       </c>
       <c r="D101" t="n">
-        <v>0.2286</v>
+        <v>0.419</v>
       </c>
       <c r="E101" t="n">
-        <v>0.2532</v>
+        <v>0.66</v>
       </c>
       <c r="F101" t="n">
-        <v>0.2575</v>
+        <v>0.6523</v>
       </c>
       <c r="G101" t="n">
-        <v>0.208</v>
+        <v>0.5174</v>
       </c>
       <c r="H101" t="n">
-        <v>0.292</v>
+        <v>0.3902</v>
       </c>
     </row>
     <row r="102">
@@ -2764,16 +2764,16 @@
       </c>
       <c r="B102" t="inlineStr"/>
       <c r="C102" t="n">
-        <v>0.2424</v>
+        <v>0.2438</v>
       </c>
       <c r="D102" t="n">
-        <v>0.2155</v>
+        <v>0.3296</v>
       </c>
       <c r="E102" t="n">
-        <v>0.2119</v>
+        <v>0.2517</v>
       </c>
       <c r="F102" t="n">
-        <v>0.2208</v>
+        <v>0.5019</v>
       </c>
       <c r="G102" t="inlineStr"/>
       <c r="H102" t="inlineStr"/>
@@ -2787,16 +2787,16 @@
       <c r="B103" t="inlineStr"/>
       <c r="C103" t="inlineStr"/>
       <c r="D103" t="n">
-        <v>0.2837</v>
+        <v>0.5538999999999999</v>
       </c>
       <c r="E103" t="n">
-        <v>0.2878</v>
+        <v>0.5784</v>
       </c>
       <c r="F103" t="n">
-        <v>0.3127</v>
+        <v>0.5474</v>
       </c>
       <c r="G103" t="n">
-        <v>0.3031</v>
+        <v>0.7608</v>
       </c>
       <c r="H103" t="inlineStr"/>
     </row>
@@ -2808,19 +2808,19 @@
       </c>
       <c r="B104" t="inlineStr"/>
       <c r="C104" t="n">
-        <v>0.2197</v>
+        <v>0.3329</v>
       </c>
       <c r="D104" t="n">
-        <v>0.2233</v>
+        <v>0.2766</v>
       </c>
       <c r="E104" t="n">
-        <v>0.239</v>
+        <v>0.2879</v>
       </c>
       <c r="F104" t="n">
-        <v>0.2258</v>
+        <v>0.5759</v>
       </c>
       <c r="G104" t="n">
-        <v>0.2084</v>
+        <v>0.3172</v>
       </c>
       <c r="H104" t="inlineStr"/>
     </row>
@@ -2832,19 +2832,19 @@
       </c>
       <c r="B105" t="inlineStr"/>
       <c r="C105" t="n">
-        <v>0.2787</v>
+        <v>0.5308</v>
       </c>
       <c r="D105" t="n">
-        <v>0.2003</v>
+        <v>0.3779</v>
       </c>
       <c r="E105" t="n">
-        <v>0.5021</v>
+        <v>0.7712</v>
       </c>
       <c r="F105" t="n">
-        <v>0.202</v>
+        <v>0.3184</v>
       </c>
       <c r="G105" t="n">
-        <v>0.2036</v>
+        <v>0.4247</v>
       </c>
       <c r="H105" t="inlineStr"/>
     </row>
@@ -2855,22 +2855,22 @@
         </is>
       </c>
       <c r="B106" t="n">
-        <v>0.2232</v>
+        <v>0.4221</v>
       </c>
       <c r="C106" t="n">
-        <v>0.2063</v>
+        <v>0.3655</v>
       </c>
       <c r="D106" t="n">
-        <v>0.2646</v>
+        <v>0.4027</v>
       </c>
       <c r="E106" t="n">
-        <v>0.2732</v>
+        <v>0.5467</v>
       </c>
       <c r="F106" t="n">
-        <v>0.2285</v>
+        <v>0.5435</v>
       </c>
       <c r="G106" t="n">
-        <v>0.314</v>
+        <v>0.3949</v>
       </c>
       <c r="H106" t="inlineStr"/>
     </row>
@@ -2882,16 +2882,16 @@
       </c>
       <c r="B107" t="inlineStr"/>
       <c r="C107" t="n">
-        <v>0.2409</v>
+        <v>0.5836</v>
       </c>
       <c r="D107" t="n">
-        <v>0.45</v>
+        <v>0.6933</v>
       </c>
       <c r="E107" t="n">
-        <v>0.3458</v>
+        <v>0.5413</v>
       </c>
       <c r="F107" t="n">
-        <v>0.3317</v>
+        <v>0.511</v>
       </c>
       <c r="G107" t="inlineStr"/>
       <c r="H107" t="inlineStr"/>
@@ -2904,19 +2904,19 @@
       </c>
       <c r="B108" t="inlineStr"/>
       <c r="C108" t="n">
-        <v>0.3245</v>
+        <v>0.5201</v>
       </c>
       <c r="D108" t="n">
-        <v>0.3245</v>
+        <v>0.5201</v>
       </c>
       <c r="E108" t="n">
-        <v>0.3633</v>
+        <v>0.5506</v>
       </c>
       <c r="F108" t="n">
-        <v>0.2933</v>
+        <v>0.4504</v>
       </c>
       <c r="G108" t="n">
-        <v>0.226</v>
+        <v>0.593</v>
       </c>
       <c r="H108" t="inlineStr"/>
     </row>
@@ -2928,19 +2928,19 @@
       </c>
       <c r="B109" t="inlineStr"/>
       <c r="C109" t="n">
-        <v>0.2086</v>
+        <v>0.5994</v>
       </c>
       <c r="D109" t="n">
-        <v>0.2617</v>
+        <v>0.5037</v>
       </c>
       <c r="E109" t="n">
-        <v>0.2295</v>
+        <v>0.5694</v>
       </c>
       <c r="F109" t="n">
-        <v>0.428</v>
+        <v>0.5799</v>
       </c>
       <c r="G109" t="n">
-        <v>0.2152</v>
+        <v>0.4342</v>
       </c>
       <c r="H109" t="inlineStr"/>
     </row>
@@ -2953,16 +2953,16 @@
       <c r="B110" t="inlineStr"/>
       <c r="C110" t="inlineStr"/>
       <c r="D110" t="n">
-        <v>0.2029</v>
+        <v>0.5207000000000001</v>
       </c>
       <c r="E110" t="n">
-        <v>0.2933</v>
+        <v>0.7302</v>
       </c>
       <c r="F110" t="n">
-        <v>0.2805</v>
+        <v>0.6048</v>
       </c>
       <c r="G110" t="n">
-        <v>0.2546</v>
+        <v>0.5058</v>
       </c>
       <c r="H110" t="inlineStr"/>
     </row>
@@ -2973,22 +2973,22 @@
         </is>
       </c>
       <c r="B111" t="n">
-        <v>0.2759</v>
+        <v>0.5184</v>
       </c>
       <c r="C111" t="n">
-        <v>0.259</v>
+        <v>0.5399</v>
       </c>
       <c r="D111" t="n">
-        <v>0.2484</v>
+        <v>0.4148</v>
       </c>
       <c r="E111" t="n">
-        <v>0.2639</v>
+        <v>0.445</v>
       </c>
       <c r="F111" t="n">
-        <v>0.3399</v>
+        <v>0.5249</v>
       </c>
       <c r="G111" t="n">
-        <v>0.2387</v>
+        <v>0.3194</v>
       </c>
       <c r="H111" t="inlineStr"/>
     </row>
@@ -3002,13 +3002,13 @@
         <v>0.4539</v>
       </c>
       <c r="C112" t="n">
-        <v>0.2976</v>
+        <v>0.6768</v>
       </c>
       <c r="D112" t="n">
         <v>0.4412</v>
       </c>
       <c r="E112" t="n">
-        <v>0.2192</v>
+        <v>0.5528</v>
       </c>
       <c r="F112" t="n">
         <v>0.4449</v>
@@ -3026,7 +3026,7 @@
       </c>
       <c r="B113" t="inlineStr"/>
       <c r="C113" t="n">
-        <v>0.2398</v>
+        <v>0.2673</v>
       </c>
       <c r="D113" t="n">
         <v>0.213</v>
@@ -3035,7 +3035,7 @@
         <v>0.2581</v>
       </c>
       <c r="F113" t="n">
-        <v>0.2732</v>
+        <v>0.3311</v>
       </c>
       <c r="G113" t="inlineStr"/>
       <c r="H113" t="inlineStr"/>
@@ -3048,7 +3048,7 @@
       </c>
       <c r="B114" t="inlineStr"/>
       <c r="C114" t="n">
-        <v>0.2828</v>
+        <v>0.5145</v>
       </c>
       <c r="D114" t="n">
         <v>0.2907</v>
@@ -3057,10 +3057,10 @@
         <v>0.295</v>
       </c>
       <c r="F114" t="n">
-        <v>0.2239</v>
+        <v>0.4578</v>
       </c>
       <c r="G114" t="n">
-        <v>0.3151</v>
+        <v>0.4678</v>
       </c>
       <c r="H114" t="inlineStr"/>
     </row>
@@ -3075,16 +3075,16 @@
         <v>0.2644</v>
       </c>
       <c r="D115" t="n">
-        <v>0.2043</v>
+        <v>0.3541</v>
       </c>
       <c r="E115" t="n">
-        <v>0.2437</v>
+        <v>0.296</v>
       </c>
       <c r="F115" t="n">
-        <v>0.2124</v>
+        <v>0.4528</v>
       </c>
       <c r="G115" t="n">
-        <v>0.2124</v>
+        <v>0.3326</v>
       </c>
       <c r="H115" t="inlineStr"/>
     </row>
@@ -3096,19 +3096,19 @@
       </c>
       <c r="B116" t="inlineStr"/>
       <c r="C116" t="n">
-        <v>0.2625</v>
+        <v>0.627</v>
       </c>
       <c r="D116" t="n">
-        <v>0.273</v>
+        <v>0.5564</v>
       </c>
       <c r="E116" t="n">
-        <v>0.2487</v>
+        <v>0.5419</v>
       </c>
       <c r="F116" t="n">
-        <v>0.2578</v>
+        <v>0.6183999999999999</v>
       </c>
       <c r="G116" t="n">
-        <v>0.2464</v>
+        <v>0.5093</v>
       </c>
       <c r="H116" t="inlineStr"/>
     </row>
@@ -3120,19 +3120,19 @@
       </c>
       <c r="B117" t="inlineStr"/>
       <c r="C117" t="n">
-        <v>0.282</v>
+        <v>0.4796</v>
       </c>
       <c r="D117" t="n">
-        <v>0.2894</v>
+        <v>0.3338</v>
       </c>
       <c r="E117" t="n">
-        <v>0.2499</v>
+        <v>0.3838</v>
       </c>
       <c r="F117" t="n">
-        <v>0.248</v>
+        <v>0.4371</v>
       </c>
       <c r="G117" t="n">
-        <v>0.2674</v>
+        <v>0.3908</v>
       </c>
       <c r="H117" t="inlineStr"/>
     </row>
@@ -3143,16 +3143,16 @@
         </is>
       </c>
       <c r="B118" t="n">
-        <v>0.2466</v>
+        <v>0.6199</v>
       </c>
       <c r="C118" t="n">
-        <v>0.2147</v>
+        <v>0.5867</v>
       </c>
       <c r="D118" t="n">
-        <v>0.2535</v>
+        <v>0.5629</v>
       </c>
       <c r="E118" t="n">
-        <v>0.3715</v>
+        <v>0.5835</v>
       </c>
       <c r="F118" t="n">
         <v>0.4588</v>
@@ -3168,10 +3168,10 @@
       </c>
       <c r="B119" t="inlineStr"/>
       <c r="C119" t="n">
-        <v>0.2392</v>
+        <v>0.2641</v>
       </c>
       <c r="D119" t="n">
-        <v>0.2132</v>
+        <v>0.2811</v>
       </c>
       <c r="E119" t="n">
         <v>0.5042</v>
@@ -3192,16 +3192,16 @@
       </c>
       <c r="B120" t="inlineStr"/>
       <c r="C120" t="n">
-        <v>0.3202</v>
+        <v>0.3567</v>
       </c>
       <c r="D120" t="n">
-        <v>0.266</v>
+        <v>0.3185</v>
       </c>
       <c r="E120" t="n">
-        <v>0.2191</v>
+        <v>0.3643</v>
       </c>
       <c r="F120" t="n">
-        <v>0.2056</v>
+        <v>0.3018</v>
       </c>
       <c r="G120" t="inlineStr"/>
       <c r="H120" t="inlineStr"/>
@@ -3216,10 +3216,10 @@
       <c r="C121" t="inlineStr"/>
       <c r="D121" t="inlineStr"/>
       <c r="E121" t="n">
-        <v>0.2618</v>
+        <v>0.6478</v>
       </c>
       <c r="F121" t="n">
-        <v>0.2642</v>
+        <v>0.5523</v>
       </c>
       <c r="G121" t="inlineStr"/>
       <c r="H121" t="inlineStr"/>
@@ -3237,10 +3237,10 @@
         <v>0.2977</v>
       </c>
       <c r="F122" t="n">
-        <v>0.2192</v>
+        <v>0.3016</v>
       </c>
       <c r="G122" t="n">
-        <v>0.2311</v>
+        <v>0.3923</v>
       </c>
       <c r="H122" t="inlineStr"/>
     </row>
@@ -3254,13 +3254,13 @@
       <c r="C123" t="inlineStr"/>
       <c r="D123" t="inlineStr"/>
       <c r="E123" t="n">
-        <v>0.2067</v>
+        <v>0.3446</v>
       </c>
       <c r="F123" t="n">
         <v>0.4134</v>
       </c>
       <c r="G123" t="n">
-        <v>0.2797</v>
+        <v>0.31</v>
       </c>
       <c r="H123" t="inlineStr"/>
     </row>
@@ -3274,13 +3274,13 @@
       <c r="C124" t="inlineStr"/>
       <c r="D124" t="inlineStr"/>
       <c r="E124" t="n">
-        <v>0.2779</v>
+        <v>0.3688</v>
       </c>
       <c r="F124" t="n">
-        <v>0.283</v>
+        <v>0.36</v>
       </c>
       <c r="G124" t="n">
-        <v>0.2896</v>
+        <v>0.4104</v>
       </c>
       <c r="H124" t="inlineStr"/>
     </row>
@@ -3294,13 +3294,13 @@
       <c r="C125" t="inlineStr"/>
       <c r="D125" t="inlineStr"/>
       <c r="E125" t="n">
-        <v>0.2414</v>
+        <v>0.2521</v>
       </c>
       <c r="F125" t="n">
-        <v>0.2087</v>
+        <v>0.4237</v>
       </c>
       <c r="G125" t="n">
-        <v>0.21</v>
+        <v>0.2606</v>
       </c>
       <c r="H125" t="inlineStr"/>
     </row>
@@ -3312,19 +3312,19 @@
       </c>
       <c r="B126" t="inlineStr"/>
       <c r="C126" t="n">
-        <v>0.3267</v>
+        <v>0.451</v>
       </c>
       <c r="D126" t="n">
-        <v>0.336</v>
+        <v>0.4571</v>
       </c>
       <c r="E126" t="n">
-        <v>0.2001</v>
+        <v>0.4971</v>
       </c>
       <c r="F126" t="n">
-        <v>0.2784</v>
+        <v>0.3966</v>
       </c>
       <c r="G126" t="n">
-        <v>0.2221</v>
+        <v>0.2983</v>
       </c>
       <c r="H126" t="inlineStr"/>
     </row>
@@ -3336,22 +3336,22 @@
       </c>
       <c r="B127" t="inlineStr"/>
       <c r="C127" t="n">
-        <v>0.239</v>
+        <v>0.5846</v>
       </c>
       <c r="D127" t="n">
-        <v>0.2356</v>
+        <v>0.321</v>
       </c>
       <c r="E127" t="n">
-        <v>0.4497</v>
+        <v>0.6928</v>
       </c>
       <c r="F127" t="n">
-        <v>0.2309</v>
+        <v>0.5047</v>
       </c>
       <c r="G127" t="n">
-        <v>0.3497</v>
+        <v>0.351</v>
       </c>
       <c r="H127" t="n">
-        <v>0.2911</v>
+        <v>0.3676</v>
       </c>
     </row>
     <row r="128">
@@ -3363,7 +3363,7 @@
       <c r="B128" t="inlineStr"/>
       <c r="C128" t="inlineStr"/>
       <c r="D128" t="n">
-        <v>0.238</v>
+        <v>0.4859</v>
       </c>
       <c r="E128" t="n">
         <v>0.2829</v>
@@ -3382,16 +3382,16 @@
       </c>
       <c r="B129" t="inlineStr"/>
       <c r="C129" t="n">
-        <v>0.2233</v>
+        <v>0.3164</v>
       </c>
       <c r="D129" t="n">
-        <v>0.4986</v>
+        <v>0.653</v>
       </c>
       <c r="E129" t="n">
-        <v>0.5665</v>
+        <v>0.7239</v>
       </c>
       <c r="F129" t="n">
-        <v>0.4813</v>
+        <v>0.6245000000000001</v>
       </c>
       <c r="G129" t="inlineStr"/>
       <c r="H129" t="inlineStr"/>
@@ -3404,19 +3404,19 @@
       </c>
       <c r="B130" t="inlineStr"/>
       <c r="C130" t="n">
-        <v>0.2174</v>
+        <v>0.2423</v>
       </c>
       <c r="D130" t="n">
-        <v>0.2695</v>
+        <v>0.2983</v>
       </c>
       <c r="E130" t="n">
-        <v>0.2091</v>
+        <v>0.2816</v>
       </c>
       <c r="F130" t="n">
-        <v>0.2339</v>
+        <v>0.4518</v>
       </c>
       <c r="G130" t="n">
-        <v>0.2385</v>
+        <v>0.2843</v>
       </c>
       <c r="H130" t="inlineStr"/>
     </row>
@@ -3429,16 +3429,16 @@
       <c r="B131" t="inlineStr"/>
       <c r="C131" t="inlineStr"/>
       <c r="D131" t="n">
-        <v>0.243</v>
+        <v>0.4115</v>
       </c>
       <c r="E131" t="n">
-        <v>0.367</v>
+        <v>0.4977</v>
       </c>
       <c r="F131" t="n">
         <v>0.2914</v>
       </c>
       <c r="G131" t="n">
-        <v>0.2687</v>
+        <v>0.6412</v>
       </c>
       <c r="H131" t="inlineStr"/>
     </row>
@@ -3451,19 +3451,19 @@
       <c r="B132" t="inlineStr"/>
       <c r="C132" t="inlineStr"/>
       <c r="D132" t="n">
-        <v>0.308</v>
+        <v>0.3772</v>
       </c>
       <c r="E132" t="n">
-        <v>0.224</v>
+        <v>0.2555</v>
       </c>
       <c r="F132" t="n">
-        <v>0.22</v>
+        <v>0.4055</v>
       </c>
       <c r="G132" t="n">
-        <v>0.2298</v>
+        <v>0.486</v>
       </c>
       <c r="H132" t="n">
-        <v>0.258</v>
+        <v>0.4156</v>
       </c>
     </row>
     <row r="133">
@@ -3478,7 +3478,7 @@
       <c r="E133" t="inlineStr"/>
       <c r="F133" t="inlineStr"/>
       <c r="G133" t="n">
-        <v>0.2014</v>
+        <v>0.2794</v>
       </c>
       <c r="H133" t="n">
         <v>0.3119</v>
@@ -3492,22 +3492,22 @@
       </c>
       <c r="B134" t="inlineStr"/>
       <c r="C134" t="n">
-        <v>0.2072</v>
+        <v>0.3226</v>
       </c>
       <c r="D134" t="n">
-        <v>0.2361</v>
+        <v>0.3051</v>
       </c>
       <c r="E134" t="n">
-        <v>0.2007</v>
+        <v>0.266</v>
       </c>
       <c r="F134" t="n">
-        <v>0.2616</v>
+        <v>0.3078</v>
       </c>
       <c r="G134" t="n">
-        <v>0.2488</v>
+        <v>0.3528</v>
       </c>
       <c r="H134" t="n">
-        <v>0.2205</v>
+        <v>0.4291</v>
       </c>
     </row>
     <row r="135">
@@ -3518,22 +3518,22 @@
       </c>
       <c r="B135" t="inlineStr"/>
       <c r="C135" t="n">
-        <v>0.2165</v>
+        <v>0.3358</v>
       </c>
       <c r="D135" t="n">
-        <v>0.3412</v>
+        <v>0.3437</v>
       </c>
       <c r="E135" t="n">
-        <v>0.2165</v>
+        <v>0.3687</v>
       </c>
       <c r="F135" t="n">
-        <v>0.227</v>
+        <v>0.3221</v>
       </c>
       <c r="G135" t="n">
-        <v>0.2713</v>
+        <v>0.3323</v>
       </c>
       <c r="H135" t="n">
-        <v>0.28</v>
+        <v>0.4486</v>
       </c>
     </row>
     <row r="136">
@@ -3544,22 +3544,22 @@
       </c>
       <c r="B136" t="inlineStr"/>
       <c r="C136" t="n">
-        <v>0.2712</v>
+        <v>0.5139</v>
       </c>
       <c r="D136" t="n">
-        <v>0.2297</v>
+        <v>0.3746</v>
       </c>
       <c r="E136" t="n">
-        <v>0.2439</v>
+        <v>0.3714</v>
       </c>
       <c r="F136" t="n">
-        <v>0.2655</v>
+        <v>0.4078</v>
       </c>
       <c r="G136" t="n">
-        <v>0.2706</v>
+        <v>0.3987</v>
       </c>
       <c r="H136" t="n">
-        <v>0.2077</v>
+        <v>0.3213</v>
       </c>
     </row>
     <row r="137">
@@ -3572,16 +3572,16 @@
       <c r="C137" t="inlineStr"/>
       <c r="D137" t="inlineStr"/>
       <c r="E137" t="n">
-        <v>0.2697</v>
+        <v>0.4024</v>
       </c>
       <c r="F137" t="n">
-        <v>0.2849</v>
+        <v>0.3684</v>
       </c>
       <c r="G137" t="n">
-        <v>0.2312</v>
+        <v>0.4273</v>
       </c>
       <c r="H137" t="n">
-        <v>0.2378</v>
+        <v>0.6832</v>
       </c>
     </row>
     <row r="138">
@@ -3591,22 +3591,22 @@
         </is>
       </c>
       <c r="B138" t="n">
-        <v>0.2386</v>
+        <v>0.5227000000000001</v>
       </c>
       <c r="C138" t="n">
-        <v>0.3036</v>
+        <v>0.4662</v>
       </c>
       <c r="D138" t="n">
-        <v>0.2021</v>
+        <v>0.384</v>
       </c>
       <c r="E138" t="n">
-        <v>0.2356</v>
+        <v>0.4064</v>
       </c>
       <c r="F138" t="n">
-        <v>0.3497</v>
+        <v>0.6251</v>
       </c>
       <c r="G138" t="n">
-        <v>0.2994</v>
+        <v>0.4598</v>
       </c>
       <c r="H138" t="inlineStr"/>
     </row>
@@ -3617,22 +3617,22 @@
         </is>
       </c>
       <c r="B139" t="n">
-        <v>0.252</v>
+        <v>0.6355</v>
       </c>
       <c r="C139" t="n">
-        <v>0.326</v>
+        <v>0.482</v>
       </c>
       <c r="D139" t="n">
-        <v>0.2233</v>
+        <v>0.4467</v>
       </c>
       <c r="E139" t="n">
-        <v>0.2446</v>
+        <v>0.5608</v>
       </c>
       <c r="F139" t="n">
-        <v>0.2401</v>
+        <v>0.509</v>
       </c>
       <c r="G139" t="n">
-        <v>0.3081</v>
+        <v>0.6131</v>
       </c>
       <c r="H139" t="inlineStr"/>
     </row>
@@ -3645,16 +3645,16 @@
       <c r="B140" t="inlineStr"/>
       <c r="C140" t="inlineStr"/>
       <c r="D140" t="n">
-        <v>0.2047</v>
+        <v>0.4052</v>
       </c>
       <c r="E140" t="n">
-        <v>0.2796</v>
+        <v>0.4034</v>
       </c>
       <c r="F140" t="n">
-        <v>0.2239</v>
+        <v>0.5657</v>
       </c>
       <c r="G140" t="n">
-        <v>0.2229</v>
+        <v>0.4296</v>
       </c>
       <c r="H140" t="inlineStr"/>
     </row>
@@ -3667,16 +3667,16 @@
       <c r="B141" t="inlineStr"/>
       <c r="C141" t="inlineStr"/>
       <c r="D141" t="n">
-        <v>0.4272</v>
+        <v>0.7213000000000001</v>
       </c>
       <c r="E141" t="n">
-        <v>0.2523</v>
+        <v>0.5933</v>
       </c>
       <c r="F141" t="n">
-        <v>0.3194</v>
+        <v>0.5009</v>
       </c>
       <c r="G141" t="n">
-        <v>0.4023</v>
+        <v>0.6414</v>
       </c>
       <c r="H141" t="inlineStr"/>
     </row>
@@ -3687,22 +3687,22 @@
         </is>
       </c>
       <c r="B142" t="n">
-        <v>0.5078</v>
+        <v>0.8575</v>
       </c>
       <c r="C142" t="n">
-        <v>0.4654</v>
+        <v>0.7857</v>
       </c>
       <c r="D142" t="n">
-        <v>0.4502</v>
+        <v>0.7602</v>
       </c>
       <c r="E142" t="n">
-        <v>0.403</v>
+        <v>0.6804</v>
       </c>
       <c r="F142" t="n">
-        <v>0.3203</v>
+        <v>0.5377999999999999</v>
       </c>
       <c r="G142" t="n">
-        <v>0.5251</v>
+        <v>0.8866000000000001</v>
       </c>
       <c r="H142" t="inlineStr"/>
     </row>
@@ -3716,13 +3716,13 @@
       <c r="C143" t="inlineStr"/>
       <c r="D143" t="inlineStr"/>
       <c r="E143" t="n">
-        <v>0.2561</v>
+        <v>0.5762</v>
       </c>
       <c r="F143" t="n">
-        <v>0.2169</v>
+        <v>0.4074</v>
       </c>
       <c r="G143" t="n">
-        <v>0.2105</v>
+        <v>0.471</v>
       </c>
       <c r="H143" t="n">
         <v>0.3785</v>
@@ -3737,16 +3737,16 @@
       <c r="B144" t="inlineStr"/>
       <c r="C144" t="inlineStr"/>
       <c r="D144" t="n">
-        <v>0.2678</v>
+        <v>0.5132</v>
       </c>
       <c r="E144" t="n">
-        <v>0.2101</v>
+        <v>0.3397</v>
       </c>
       <c r="F144" t="n">
-        <v>0.2329</v>
+        <v>0.4651</v>
       </c>
       <c r="G144" t="n">
-        <v>0.2276</v>
+        <v>0.3574</v>
       </c>
       <c r="H144" t="inlineStr"/>
     </row>
@@ -3760,13 +3760,13 @@
       <c r="C145" t="inlineStr"/>
       <c r="D145" t="inlineStr"/>
       <c r="E145" t="n">
-        <v>0.2793</v>
+        <v>0.5213</v>
       </c>
       <c r="F145" t="n">
-        <v>0.2342</v>
+        <v>0.3985</v>
       </c>
       <c r="G145" t="n">
-        <v>0.2231</v>
+        <v>0.4164</v>
       </c>
       <c r="H145" t="inlineStr"/>
     </row>
@@ -3779,16 +3779,16 @@
       <c r="B146" t="inlineStr"/>
       <c r="C146" t="inlineStr"/>
       <c r="D146" t="n">
-        <v>0.2379</v>
+        <v>0.4532</v>
       </c>
       <c r="E146" t="n">
-        <v>0.2232</v>
+        <v>0.4131</v>
       </c>
       <c r="F146" t="n">
-        <v>0.2674</v>
+        <v>0.3788</v>
       </c>
       <c r="G146" t="n">
-        <v>0.2311</v>
+        <v>0.2653</v>
       </c>
       <c r="H146" t="inlineStr"/>
     </row>
@@ -3801,10 +3801,10 @@
       <c r="B147" t="inlineStr"/>
       <c r="C147" t="inlineStr"/>
       <c r="D147" t="n">
-        <v>0.3293</v>
+        <v>0.5174</v>
       </c>
       <c r="E147" t="n">
-        <v>0.2321</v>
+        <v>0.5659</v>
       </c>
       <c r="F147" t="n">
         <v>0.3799</v>
@@ -3820,16 +3820,16 @@
       </c>
       <c r="B148" t="inlineStr"/>
       <c r="C148" t="n">
-        <v>0.3316</v>
+        <v>0.381</v>
       </c>
       <c r="D148" t="n">
-        <v>0.3064</v>
+        <v>0.4606</v>
       </c>
       <c r="E148" t="n">
-        <v>0.2992</v>
+        <v>0.3482</v>
       </c>
       <c r="F148" t="n">
-        <v>0.3255</v>
+        <v>0.3666</v>
       </c>
       <c r="G148" t="inlineStr"/>
       <c r="H148" t="inlineStr"/>

</xml_diff>